<commit_message>
test: Add xai metrics
</commit_message>
<xml_diff>
--- a/experiments/cnn/CNN_Metrics.xlsx
+++ b/experiments/cnn/CNN_Metrics.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\IC\CiaAgro_FungalSpores\experiments\cnn\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub_CiaAgro\CiaAgro_FungalSpores\experiments\cnn\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA444B56-18F3-4D7D-B7CD-B9E1C794DE20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31FDEAFF-1B39-457B-A482-00B6857F9BB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5263" yWindow="2160" windowWidth="16457" windowHeight="10183" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Metrics" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="41">
   <si>
     <t>model</t>
   </si>
@@ -499,19 +499,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:T12"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="4" max="4" width="14.53515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.84375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="17.15234375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="17.140625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="14" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="11.84375" bestFit="1" customWidth="1"/>
-    <col min="11" max="12" width="11.84375" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="11.84375" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="11.84375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="12" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="11.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -573,7 +573,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="2" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>20</v>
       </c>
@@ -583,8 +583,8 @@
       <c r="C2">
         <v>0.99688473520249221</v>
       </c>
-      <c r="D2" t="s">
-        <v>3</v>
+      <c r="D2">
+        <v>0.99014270500000001</v>
       </c>
       <c r="E2">
         <v>0.984467707301655</v>
@@ -635,7 +635,7 @@
         <v>0.99881493185858183</v>
       </c>
     </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>20</v>
       </c>
@@ -645,8 +645,8 @@
       <c r="C3">
         <v>0.50040990326282997</v>
       </c>
-      <c r="D3" t="s">
-        <v>3</v>
+      <c r="D3">
+        <v>0.38539330199999999</v>
       </c>
       <c r="E3">
         <v>0.45918112388820881</v>
@@ -697,7 +697,7 @@
         <v>0.63131245836109262</v>
       </c>
     </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>23</v>
       </c>
@@ -759,7 +759,7 @@
         <v>0.99792551615133851</v>
       </c>
     </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>23</v>
       </c>
@@ -821,7 +821,7 @@
         <v>0.9287503757891572</v>
       </c>
     </row>
-    <row r="8" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>24</v>
       </c>
@@ -883,7 +883,7 @@
         <v>0.97277537277537274</v>
       </c>
     </row>
-    <row r="9" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>24</v>
       </c>
@@ -945,7 +945,7 @@
         <v>0.99585553582001185</v>
       </c>
     </row>
-    <row r="11" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>25</v>
       </c>
@@ -1007,7 +1007,7 @@
         <v>0.99753135183173691</v>
       </c>
     </row>
-    <row r="12" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>25</v>
       </c>
@@ -1077,7 +1077,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:I23"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
     <col min="2" max="4" width="11" customWidth="1"/>
@@ -1086,7 +1086,7 @@
     <col min="7" max="9" width="11" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="15.9" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>26</v>
       </c>
@@ -1100,7 +1100,7 @@
       <c r="H1" s="3"/>
       <c r="I1" s="3"/>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>28</v>
       </c>
@@ -1126,7 +1126,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>32</v>
       </c>
@@ -1152,7 +1152,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>33</v>
       </c>
@@ -1178,7 +1178,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>34</v>
       </c>
@@ -1204,7 +1204,7 @@
         <v>2369</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="15.9" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>35</v>
       </c>
@@ -1218,7 +1218,7 @@
       <c r="H7" s="3"/>
       <c r="I7" s="3"/>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>28</v>
       </c>
@@ -1244,7 +1244,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>32</v>
       </c>
@@ -1270,7 +1270,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>33</v>
       </c>
@@ -1296,7 +1296,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>34</v>
       </c>
@@ -1322,7 +1322,7 @@
         <v>4634</v>
       </c>
     </row>
-    <row r="13" spans="1:9" ht="15.9" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>37</v>
       </c>
@@ -1336,7 +1336,7 @@
       <c r="H13" s="3"/>
       <c r="I13" s="3"/>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>28</v>
       </c>
@@ -1362,7 +1362,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>32</v>
       </c>
@@ -1388,7 +1388,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>33</v>
       </c>
@@ -1414,7 +1414,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>34</v>
       </c>
@@ -1440,7 +1440,7 @@
         <v>5046</v>
       </c>
     </row>
-    <row r="19" spans="1:9" ht="15.9" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>39</v>
       </c>
@@ -1454,7 +1454,7 @@
       <c r="H19" s="3"/>
       <c r="I19" s="3"/>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>28</v>
       </c>
@@ -1480,7 +1480,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>32</v>
       </c>
@@ -1506,7 +1506,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>33</v>
       </c>
@@ -1532,7 +1532,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>34</v>
       </c>

</xml_diff>